<commit_message>
Align Day 1 deliverables with AeroVanguard AV-X9 Aetheris technical blueprint (AVT-AETH-2026-X9)
</commit_message>
<xml_diff>
--- a/Day 1/P02_Initial_Requirements_Register.xlsx
+++ b/Day 1/P02_Initial_Requirements_Register.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_References" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements_Register'!$A$1:$L$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements_Register'!$A$1:$L$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,12 +51,6 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="008A6D3B"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
@@ -79,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -102,12 +96,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,9 +171,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -209,18 +197,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -230,14 +213,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -608,16 +591,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -695,7 +678,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>The system shall capture and hardware-synchronize daylight optical CMOS video and uncooled Long-Wave Infrared (LWIR) bolometer thermal video streams over multi-lane MIPI-CSI Gen3 camera buses.</t>
+          <t>The system shall capture and hardware-synchronize daylight 4K Sony CMOS optical video and 640x512 uncooled FLIR Boson thermal video streams via MIPI-CSI 4-Lane Gen3 camera interfaces.</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -710,17 +693,17 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Section 7 (Module 02), Section 8.2 (p. 8, 9)</t>
+          <t>Section 1.2, Section 7 (Module 02), Section 8.1 (p. 1, 7, 8)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Module 02 provides stabilized day/night surveillance and target acquisition through fog and dust via high-speed MIPI-CSI dual-stream video.</t>
+          <t>Module 02 (OptiSight) integrates 4K Sony CMOS and 640x512 FLIR Boson thermal lens outputting dual feeds over MIPI-CSI.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -740,12 +723,12 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Optical CMOS resolution (e.g. 4K/1080p), LWIR bolometer resolution (e.g. 640x512), and frame rates (FPS) not quantified in technical overview.</t>
+          <t>Optical CMOS field-of-view (FOV) and zoom lens magnification ratios not stated in blueprint.</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Feeds directly into Module 03 (EDGE-AI) via Layer A.</t>
+          <t>Part of Module 02 (OptiSight) and Layer A.</t>
         </is>
       </c>
     </row>
@@ -757,7 +740,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>The system shall ingest real-time distance measurements and obstacle point clouds from an onboard lightweight micro-LiDAR sensor over a dedicated high-speed serial bus.</t>
+          <t>The system shall capture and stream 16-bit IQ complex radar samples from an onboard micro-Ground Penetrating Radar (GPR) antenna over USB 3.0 / PCIe x2 into dedicated DSP priority buffers to detect buried tactical targets.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -767,22 +750,22 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Perception &amp; Ingress</t>
+          <t>Subsurface Radar Sensing</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Section 3.1, Section 6.2, Section 7 (Module 01) (p. 4, 7, 8)</t>
+          <t>Section 3.2, Section 8.1 (p. 3, 8)</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Micro-LiDAR range data serves as an active input for terrain elevation modeling, obstacle avoidance, and VIO drift correction.</t>
+          <t>Section 8.1 specifies USB 3.0 / PCIe x2 interface transferring 16-bit IQ complex samples with dedicated DSP priority ring buffers.</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -795,19 +778,19 @@
           <t>Test</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Micro-LiDAR update rate (Hz), maximum operating range (meters), angular field of view, and exact physical interface protocol not stated.</t>
+          <t>Center frequency and soil/ice penetration depth specifications not defined.</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>Shared between Module 01 (VIO-NAV) and Module 02.</t>
+          <t>Layer A sensory ingress feeding Layer C DSP pipeline.</t>
         </is>
       </c>
     </row>
@@ -819,7 +802,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>The system shall ingest synchronized acoustic air pressure signals from a 4-channel microphone array and execute Time-Difference-of-Arrival (TDoA) algorithms to calculate bearing vectors to acoustic impulse noises.</t>
+          <t>The system shall ingest acoustic air pressure signals from a 4-channel microphone array and execute Time-Difference-of-Arrival (TDoA) algorithms to calculate directional bearing estimates to acoustic impulse noises.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -834,17 +817,17 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 5), Section 7 (Module 04), Section 8.2 (p. 5, 8, 9)</t>
+          <t>Section 1.2, Section 4, Section 7 (Module 04) (p. 1, 4, 7)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Module 04 evaluates Time-Difference-of-Arrival (TDoA) acoustic localization from a 4-channel microphone array over high-speed SPI/USB 3.0 audio PDM arrays.</t>
+          <t>Module 04 evaluates Time-Difference-of-Arrival acoustic localization from a 4-channel microphone array.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -857,19 +840,19 @@
           <t>Demonstration</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Acoustic sampling rate, frequency response band, minimum detection range, and angular bearing accuracy threshold missing.</t>
+          <t>Acoustic sampling frequency and minimum impulse detection sensitivity not specified.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Part of Module 04 (EW-DSP) and Layer A.</t>
+          <t>Part of Module 04 (SpectraSense).</t>
         </is>
       </c>
     </row>
@@ -881,7 +864,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>The system shall capture and condition subsurface radar echo signals from an onboard micro-Ground Penetrating Radar (GPR) antenna to detect subsurface anomalies and buried tactical targets.</t>
+          <t>The system shall maintain real-time 6-DOF vehicle pose and velocity estimation in GNSS-denied environments by fusing dual stereo visual odometry, tactical-grade 200Hz IMU angular rates, and onboard DEM terrain matching via extended Kalman filtering (EKF3).</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -891,22 +874,22 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Subsurface Sensing &amp; DSP</t>
+          <t>Navigation &amp; Autonomy</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 8), Section 7 (Module 04), Section 8.2 (p. 5, 8, 9)</t>
+          <t>Section 1.1, Section 2.2, Section 7 (Module 01) (p. 1, 2, 7)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Module 04 processes 16-bit IQ samples from a micro-GPR antenna routed via high-speed SPI/USB 3.0 to image subsurface targets.</t>
+          <t>AetherNav VIO Matrix combines dual stereo visual odometry, tactical-grade 200Hz IMU units, and DEM terrain matching for zero-drift positioning.</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -919,19 +902,19 @@
           <t>Test</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>GPR center frequency, radar bandwidth, maximum penetration depth across ice/snow/dry soil, and spatial resolution undefined.</t>
+          <t>DEM database spatial resolution (e.g. 1m vs 5m grid) not quantified.</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Layer A sensory ingress feeding Layer C DSP thread.</t>
+          <t>Module 01 (AetherNav) and Layer B.</t>
         </is>
       </c>
     </row>
@@ -943,7 +926,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>The system shall ingest environmental transducer telemetry from onboard airborne CBRN sensors to detect and map airborne chemical, biological, radiological, and nuclear hazard plumes.</t>
+          <t>The system shall execute real-time attitude PID loops, waypoint navigation, and autonomous trajectory control via VanguardFlight OS combined with PX4 flight control firmware on dual-redundant STM32H7 microcontrollers.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -953,22 +936,22 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Environmental Sensing &amp; CBRN</t>
+          <t>Flight Control &amp; Avionics</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Section 3.1, Section 4 (Domain 8), Section 7 (Module 02) (p. 4, 5, 8)</t>
+          <t>Section 1.1, Section 1.2, Section 6.2 (p. 1, 6)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Digital CBRN sniffers provide airborne hazard-mapping data within the multi-modal sensor payload suite.</t>
+          <t>VanguardFlight OS combines a proprietary real-time microkernel OS with PX4 flight control loops running on dual STM32H7 MCUs.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -981,19 +964,19 @@
           <t>Demonstration</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Target chemical/radiological detection thresholds, sensor response latency, and MAVLink telemetry reporting packet format unspecified.</t>
+          <t>Bank angle limits, maximum climb/descent rates, and autonomous return-to-base triggers need specification in SSRD.</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Belongs to Layer A / Module 02.</t>
+          <t>Layer B flight avionics stack.</t>
         </is>
       </c>
     </row>
@@ -1005,7 +988,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>The system shall maintain real-time 6-DOF vehicle pose, velocity, and altitude estimation in satellite-jammed airspace by fusing high-rate IMU angular rates with Visual-Inertial Odometry (VIO) and onboard Digital Elevation Models (DEM).</t>
+          <t>The system shall execute lightweight YOLOv8 neural network models directly onboard the Nvidia Jetson Orin Industrial SOM to extract tactical targets and generate bounding boxes from synchronized video streams.</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -1015,22 +998,22 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Navigation &amp; Autonomy</t>
+          <t>Edge AI &amp; Vision</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Section 2.2 (Obj 1), Section 7 (Module 01), Section 8.2 (p. 3, 8, 9)</t>
+          <t>Section 4 (Engineering Domains), Section 7 (Module 03) (p. 4, 7)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Module 01 maintains continuous, drift-bounded 6-DOF kinematic state estimation in contested airspace without cumulative drift.</t>
+          <t>Deep Learning domain explicitly deploys lightweight YOLOv8 and vision transformer neural models for real-time edge object extraction.</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -1040,7 +1023,7 @@
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Demonstration</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1050,12 +1033,12 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>IMU sampling frequency, camera tracking framerate, DEM grid resolution (e.g. 1m vs 5m), and Kalman filter update rates not stated.</t>
+          <t>Specific YOLOv8 variant (Nano vs Small vs Medium) and target class taxonomy not stated.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>Core GNSS-denied navigation stack (Module 01 / Layer B).</t>
+          <t>Module 03 (AeroCore) and Layer F.</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1050,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>The system shall execute real-time flight stabilization, attitude control, and autonomous waypoint navigation commands via custom PX4 autopilot firmware executing on a dedicated bare-metal microcontroller.</t>
+          <t>The system shall execute vision transformer neural models on onboard GPU/NPU tensor hardware to generate real-time pixel-level semantic segmentation masks of ground terrain and obstacles.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1077,22 +1060,22 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Flight Control &amp; Autonomy</t>
+          <t>Edge AI &amp; Vision</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Section 5.2 (Stage 4), Section 6.1 (Layer 2), Section 8.3 (p. 6, 7, 9)</t>
+          <t>Section 1.1, Section 4 (Engineering Domains), Section 7 (Module 03) (p. 1, 4, 7)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>PX4 real-time attitude control loops generate microsecond PWM motor speed commands and actuator servo release signals.</t>
+          <t>AeroCore Edge-AI executes real-time semantic segmentation using vision transformer neural models.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1112,12 +1095,12 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Maximum operational bank angle, climb/descent rates, and autonomous fail-safe trajectory modes need formal specification in SSRD.</t>
+          <t>Target semantic classes and minimum acceptable mIoU segmentation accuracy not defined.</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Layer B and Layer 2 firmware execution.</t>
+          <t>Module 03 (AeroCore) and Layer F.</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1112,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>The system shall execute deep neural network inference directly on onboard heterogeneous computing hardware (GPU/NPU/DSP) to generate real-time pixel-level semantic segmentation masks of terrain and tactical obstacles.</t>
+          <t>The system shall perform comparative neural inference between live video streams and onboard historical terrain embeddings to automatically detect and flag ground modifications, fortifications, or vehicle tracks.</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1139,22 +1122,22 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Edge AI &amp; Vision</t>
+          <t>Edge AI &amp; Intelligence</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Section 2.2 (Obj 2), Section 6.3, Section 7 (Module 03) (p. 3, 7, 8)</t>
+          <t>Section 1.1, Section 2.2, Section 7 (Module 03) (p. 1, 2, 7)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Executes zero-cloud, pixel-level semantic segmentation using PyTorch models exported to ONNX and compiled via TensorRT for INT8 quantization.</t>
+          <t>AeroCore executes real-time optical change detection and temporal target extraction onboard.</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -1174,12 +1157,12 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Target semantic class taxonomy (e.g. roads, vehicles, tree cover, snow), target inference FPS, and minimum mIoU accuracy threshold undefined.</t>
+          <t>Historical embedding geo-referencing format and minimum detectable disturbance dimension not defined.</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Module 03 (EDGE-AI) and Layer F.</t>
+          <t>Module 03 (AeroCore) and Layer F.</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1174,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The system shall perform comparative visual inference between live video frames and onboard historical terrain embeddings to automatically detect and flag tactical terrain alterations and infrastructure changes.</t>
+          <t>The system shall scan wideband radio frequency spectrum across 10 MHz to 6 GHz using Software-Defined Radio to generate RF spectrum occupancy grids and isolate hostile radar and emitter signatures.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1201,22 +1184,22 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Edge AI &amp; Intelligence</t>
+          <t>Electronic Warfare &amp; DSP</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 1), Section 6.1 (Layer 4), Section 7 (Module 03) (p. 5, 7, 8)</t>
+          <t>Section 4 (DSP Domain), Section 7 (Module 04) (p. 4, 7)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Temporal change detection CNNs / Siamese networks isolate infrastructure changes and terrain modifications directly on the airframe.</t>
+          <t>Module 04 monitors contested spectrum, detects hostile emissions, and outputs RF spectrum occupancy grids across 10 MHz to 6 GHz.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1226,7 +1209,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Demonstration</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1236,12 +1219,12 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Historical embedding resolution, geographical tiling structure, false alarm probability, and change confidence score thresholds not defined.</t>
+          <t>Instantaneous capture bandwidth, sweep repetition time, and emitter classification library depth not specified.</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Module 03 (EDGE-AI) and Layer F.</t>
+          <t>Module 04 (SpectraSense) and Layer D.</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1236,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>The system shall execute neural super-resolution models on degraded optical and thermal video streams onboard to synthesize enhanced high-clarity intelligence imagery across smoke, dust, and haze.</t>
+          <t>The system shall modulate and transmit tactical telemetry, target coordinates, and compressed mission imagery to friendly optical ground terminals over a directional 1550nm Free-Space Optical (FSO) laser array.</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -1263,22 +1246,22 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Edge AI &amp; Vision</t>
+          <t>Optical Communications</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 1), Section 7 (Module 03) (p. 5, 8)</t>
+          <t>Section 1.1, Section 2.2, Section 7 (Module 05) (p. 1, 2, 7)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Module 03 generates super-resolved intelligence imagery directly on the airframe using optimized neural architectures.</t>
+          <t>AetherBeam Optical Link deploys a directional 1550nm FSO laser array providing jam-proof high-bandwidth data transit.</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -1298,12 +1281,12 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Upscaling factor (e.g. 2x, 4x), maximum per-frame latency budget, and output stream bitrate not quantified in source.</t>
+          <t>Laser beam divergence angle and optical ground terminal receiver aperture specifications not defined.</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Module 03 (EDGE-AI) and Layer F.</t>
+          <t>Module 05 (AetherBeam) and Layer E.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1298,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>The system shall monitor the radio frequency spectrum across 400 MHz to 6 GHz using a Software-Defined Radio (SDR) receiver to generate RF spectrum occupancy grids and extract hostile emitter signal characterization profiles.</t>
+          <t>The system shall maintain closed-loop coarse-fine laser pointing, acquisition, and tracking (PAT) using fast steering mirrors driven by 200Hz gyro coordinate vectors over RS-422 to compensate for airframe vibration and wind shear.</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1325,22 +1308,22 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Electromagnetic Warfare &amp; DSP</t>
+          <t>Optical Communications &amp; GNC</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 5), Section 7 (Module 04), Section 8.2 (p. 5, 8, 9)</t>
+          <t>Section 4 (Free-Space Optics), Section 8.1 (p. 4, 8)</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Module 04 detects hostile radio emissions, characterizes radar signatures, and outputs RF spectrum occupancy grids and emitter profiles.</t>
+          <t>High-Speed RS422 transfers 200Hz gyro coordinate vectors to closed-loop steering mirrors compensating for airframe vibration.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1350,7 +1333,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Demonstration</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1360,12 +1343,12 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Instantaneous capture bandwidth, sweep repetition interval, minimum detectable signal sensitivity (dBm), and signature library capacity not specified.</t>
+          <t>Fast steering mirror maximum angular deflection range and angular resolution not defined.</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Module 04 (EW-DSP) and Layer D.</t>
+          <t>Module 05 (AetherBeam) and Layer E.</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1360,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>The system shall modulate and transmit mission intelligence, processed imagery, and platform telemetry to friendly optical ground terminals over a narrow-beam Free-Space Optical (FSO) directional laser link.</t>
+          <t>The system shall establish and maintain secondary frequency-hopping, cryptographically encrypted SDR RF communications for command, control, and telemetry fallback when optical laser links are obscured.</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -1387,22 +1370,22 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>RF Communications</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Section 2.2 (Obj 6), Section 7 (Module 05), Section 8.2 (p. 3, 8, 9)</t>
+          <t>Section 2.2, Section 5.2 (Stage 5) (p. 2, 5)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Module 05 deploys directional Free-Space Optical (FSO) laser communications for high-bandwidth, intercept-free data transit completely immune to RF jamming.</t>
+          <t>Optical transmission is backed by encrypted SDR RF fallback channels.</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
@@ -1422,12 +1405,12 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Optical laser wavelength (e.g. 850nm / 1550nm), data throughput (Mbps/Gbps), maximum line-of-sight range, and beam divergence angle not specified.</t>
+          <t>RF frequency bands, hopping rates, and cryptographic encryption standard (e.g. AES-256) not specified.</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Module 05 (FSO-COMM) and Layer E.</t>
+          <t>Layer E communication fallback.</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1422,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>The system shall maintain closed-loop coarse-fine beam pointing, acquisition, and tracking (PAT) using gimbal coordinate offsets to sustain line-of-sight laser alignment with ground terminals under atmospheric wind shear.</t>
+          <t>The system shall compute real-time ballistic release timing based on target GPS/grid coordinates and real-time pitot wind estimates, and command the servo unlatching of the AeroDrop logistical payload pod.</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1449,22 +1432,22 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Communications &amp; GNC</t>
+          <t>Payload &amp; Effectors</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Section 5.2 (Stage 5), Section 8.2 (FSO Gimbal Interface) (p. 6, 9)</t>
+          <t>Section 7 (Module 06), Section 8.1 (p. 7, 8)</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>RS-422 serial interface transmits high-rate gyro coordinate offsets to FSO gimbal tracking motors to ensure stable link under high wind shear.</t>
+          <t>Module 06 manages precision delivery of payloads using pitot wind estimates to compute ballistic release and unlatch signals.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1484,12 +1467,12 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>PAT acquisition latency, coarse/fine gimbal angular tracking rate (deg/sec), and maximum allowable tracking jitter (microradians) not defined.</t>
+          <t>Cargo pod payload mass capacity (kg), internal volume dimensions, and delivery CEP accuracy not stated.</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Module 05 (FSO-COMM) and Layer E.</t>
+          <t>Module 06 (AeroDrop) and Layer G.</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1484,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>The system shall maintain a secondary frequency-hopping, cryptographically encrypted Software-Defined Radio (SDR) RF data link for telemetry, command, and fallback mission data transit when optical links are obscured.</t>
+          <t>The system shall cryptographically authenticate all boot steps, bootloader binaries, Vanguard-Linux OS kernels, and ROS 2 Humble nodes from silicon power-on using a hardware TPM 2.0 security enclave.</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -1511,22 +1494,22 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Cybersecurity &amp; Data Sovereignty</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Section 2.2 (Obj 6), Section 4 (Layer E), Section 7 (Module 05) (p. 3, 4, 8)</t>
+          <t>Section 1.2, Section 6.1, Section 6.2 (p. 1, 6)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Directional FSO laser link is backed by encrypted Software-Defined Radio (SDR) channels with automated fallback triggering.</t>
+          <t>Hardware TPM 2.0 enclave enforces cryptographically signed firmware boot steps and secure partitions.</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -1536,7 +1519,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Demonstration</t>
+          <t>Inspection</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1546,12 +1529,12 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>RF frequency bands, frequency hopping rate (hops/sec), RF transmit power (Watts), and failover switching hysteresis criteria not defined.</t>
+          <t>Specific TPM 2.0 silicon part and public key certificate infrastructure (PKI) hierarchy not defined.</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>Module 05 and Layer E.</t>
+          <t>Layer H (Cybersecurity Enclave).</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1546,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>The system shall calculate instantaneous ballistic release timing based on real-time estimated local wind vectors, ground velocity, and radar altitude, and actuate the mechanical unlatching of the precision cargo drop pod.</t>
+          <t>The system shall trigger irreversible hardware-enforced cryptographic flash memory wiping and instant zero-trace RAM purging upon detection of physical enclosure breach, anti-tamper sensor activation, or airframe capture.</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1573,22 +1556,22 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Payload &amp; Effectors</t>
+          <t>Cybersecurity &amp; Data Sovereignty</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Section 5.2 (Stage 4), Section 7 (Module 06), Section 8.2 (p. 6, 8, 9)</t>
+          <t>Section 1.2, Section 6.1, Section 6.2 (p. 1, 6)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Module 06 manages precision delivery of emergency logistic payloads, computing ballistic release timing and generating delivery verification logs.</t>
+          <t>Security daemon and hardware TPM 2.0 enclave enforce cryptographically enforced auto-destruct wiped keys and zero-trace RAM purging upon capture.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1598,7 +1581,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Demonstration</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1608,49 +1591,49 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Cargo pod payload mass capacity, maximum release altitude, target delivery accuracy (CEP in meters), and mechanical unlatch timing not defined.</t>
+          <t>Flash erasure execution time budget (milliseconds) and tamper sensor electrical voltage thresholds not specified.</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Module 06 (PAYLOAD-POD) and Layer G.</t>
+          <t>Layer H (Cybersecurity Enclave).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-F-016</t>
+          <t>DRAFT-P-001</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>The system shall trigger irreversible hardware-level sanitization and cryptographic flash memory erasure upon detection of unauthorized physical airframe breach, anti-tamper sensor trip, or capture.</t>
+          <t>The system VanguardFlight OS and PX4 flight control loops shall achieve deterministic inner-loop control latency of under 250 microseconds (&lt; 250 µs) on bare-metal ARM Cortex-M7 hardware.</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Cybersecurity &amp; Sovereignty</t>
+          <t>Avionics &amp; Control Timing</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Section 2.2 (Obj 7), Section 4 (Layer H), Section 5.2 (Stage 6) (p. 3, 4, 6)</t>
+          <t>Section 1.1, Section 10 (Tier 3 Exit Criteria) (p. 1, 10)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Layer H guarantees cryptographic execution and triggers zero-trace physical/flash memory erasure upon tamper or capture detection.</t>
+          <t>Explicitly mandates 'achieving deterministic latency under 250 microseconds' and Tier 3 exit criteria: 'Inner loop latency &lt; 250 µs'.</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
@@ -1670,24 +1653,24 @@
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>Sanitization completion time budget (e.g. &lt;500 ms) and anti-tamper switch electrical trigger threshold not specified.</t>
+          <t>Inner-loop latency measurement jitter window and CAN-BUS bus loading test profiles need definition.</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Layer H (Cybersecurity &amp; Data Sovereignty).</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-P-001</t>
+          <t>DRAFT-P-002</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>The system shall sustain an inner-loop communication latency of less than 1 millisecond between the real flight controller and edge compute boards during hardware-in-the-loop (HIL) real-time sensor execution.</t>
+          <t>The airframe, aerodynamics, and propulsion subsystems shall sustain operational flight at a service ceiling of up to 6,500 meters Above Mean Sea Level (AMSL).</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1697,22 +1680,22 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Avionics &amp; Middleware Timing</t>
+          <t>Aerodynamics &amp; Operating Regime</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Section 10.1 (Tier 3 Success Criteria) (p. 11)</t>
+          <t>Executive Summary (Operating Regimes) (p. 0/1)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Tier 3 validation explicitly establishes 'Inner-loop latency under 1 millisecond' as mandatory success criteria for HIL bench testing.</t>
+          <t>Explicitly specifies 'Operational ceiling 6,500m AMSL' under Project Overview Specifications.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1732,24 +1715,24 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Latency jitter tolerance, packet drop limits, and benchmark communication bus (UART vs Ethernet) over Micro-XRCE-DDS need formal test protocol.</t>
+          <t>Maximum climb rate at 6,500m AMSL and service ceiling margin not defined.</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>Numerical threshold explicitly defined in source document.</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-P-002</t>
+          <t>DRAFT-P-003</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>The system electronics, avionics, propulsion motors, and battery management circuits shall maintain uninterrupted operation under ambient environmental temperatures down to -20°C and low ambient pressure exposure.</t>
+          <t>The system flight stabilization and airframe structure shall sustain stable controlled flight under localized mountain wind shear of up to 25 meters per second (25 m/s).</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -1759,22 +1742,22 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Environmental &amp; Thermal</t>
+          <t>Aerodynamics &amp; Flight Stability</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Section 9.2 (Milestone 2), Section 10.1 (Tier 5) (p. 10, 11)</t>
+          <t>Executive Summary (Operating Regimes) (p. 0/1)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Milestone 2 mandates thermal profiling down to -20°C; Tier 5 mandates uninterrupted electronics operation under -20°C and low pressure exposure.</t>
+          <t>Explicitly specifies 'wind shear up to 25 m/s' under Project Overview Specifications.</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -1794,24 +1777,24 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>Maximum operating temperature (+50°C?), continuous operating duration at -20°C, and battery discharge retention percentage at -20°C not specified.</t>
+          <t>Maximum gust duration at 25 m/s and angular attitude excursion limits need definition.</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Numerical threshold explicitly defined in source document.</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-P-003</t>
+          <t>DRAFT-P-004</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>The system Software-Defined Radio (SDR) subsystem shall continuously cover the wideband radio frequency spectrum across the range of 400 MHz to 6 GHz.</t>
+          <t>The system electronics, avionics, brushless propulsion motors, and self-heating battery management cells shall maintain nominal operation in ambient temperatures down to -30°C.</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1821,22 +1804,22 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>RF &amp; Electronic Warfare</t>
+          <t>Environmental &amp; Thermal</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Section 7 (Module 04 Inputs) (p. 8)</t>
+          <t>Executive Summary, Section 10 (Tier 5 Exit Criteria) (p. 0/1, 10)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Module 04 explicitly specifies input as 'Wideband SDR RF antenna inputs (400 MHz to 6 GHz)'.</t>
+          <t>Specifications explicitly mandate 'temperatures down to -30°C' and Tier 5 chamber testing down to -30°C with nominal electrical draw.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1856,24 +1839,24 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Tuning step size, instantaneous FFT bandwidth, noise figure, and dynamic range across the 400 MHz–6 GHz band not specified.</t>
+          <t>Maximum high-temperature operating limit (+50°C?) and battery self-heating power consumption budget not stated.</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Numerical range explicitly defined in source document.</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-P-004</t>
+          <t>DRAFT-P-005</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>The system shall sustain sub-meter navigational drift bounds when operating exclusively on Visual-Inertial Odometry (VIO) and DEM terrain matching during deliberate GNSS-denied flight test trials.</t>
+          <t>The system AetherNav VIO Matrix shall sustain continuous drift-bounded positional accuracy with a position error of less than 0.8 meters per hour (&lt; 0.8m error per hour) during GNSS-denied flight.</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -1888,17 +1871,17 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Section 10.1 (Tier 8 Success Criteria) (p. 11)</t>
+          <t>Section 2.2, Section 10 (Tier 8 Exit Criteria) (p. 2, 10)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Tier 8 GNSS-Denied Testing explicitly specifies 'Sub-meter drift bounds sustained' as the success criteria.</t>
+          <t>Explicitly specifies 'Sustain continuous drift-bounded positional accuracy (&lt;0.8m error per hour) via VIO and DEM matching' and Tier 8 exit criteria.</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -1911,31 +1894,31 @@
           <t>Test</t>
         </is>
       </c>
-      <c r="J21" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>Clarification required on whether 'sub-meter' applies per unit time (e.g. per minute), per flight distance (e.g. per km flown), or total closed-loop mission CEP.</t>
+          <t>Statistical confidence interval (e.g. 1-sigma vs 2-sigma CEP) for the &lt;0.8m/hr metric needs formal definition.</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Recorded as Assumption ASM-ENG-004 in Task 1 Project Scope Baseline.</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-P-005</t>
+          <t>DRAFT-P-006</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The multi-lane MIPI-CSI Gen3 camera ingress interface shall transfer raw YUV, RGB, and 14-bit thermal video frames directly into edge compute memory via DMA with zero frame drops.</t>
+          <t>The AetherBeam Free-Space Optical transceiver shall deliver a jam-proof data throughput of at least 1.2 Gbps over an optical line-of-sight range of up to 18 kilometers.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1945,22 +1928,22 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Perception &amp; Compute Throughput</t>
+          <t>Optical Communications</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Section 8.2 (Interface: Vision to Edge AI) (p. 9)</t>
+          <t>Section 1.1, Section 11.2 (p. 1, 11)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Interface specification mandates 'DMA Direct Memory Access bypassing host CPU overhead; zero frame drop buffer'.</t>
+          <t>Explicitly specifies 'Directional 1550nm Free-Space Optical (FSO) laser array providing jam-proof 1.2 Gbps data throughput up to 18 km line-of-sight'.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1980,24 +1963,24 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>DMA FIFO ring buffer depth (number of frames) and maximum memory bus contention threshold under full sensor load not stated.</t>
+          <t>Optical link margin (dB) and bit error rate (BER) thresholds across 18 km in fog/snow conditions not quantified.</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Critical high-throughput hardware interface protocol.</t>
+          <t>Explicit numerical parameters in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-P-006</t>
+          <t>DRAFT-P-007</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>The real-time flight control subsystem shall execute inner attitude stabilization loops and sensor bus management on dedicated 32-bit automotive/aerospace microcontrollers (STM32 series).</t>
+          <t>The AeroCore Edge-AI subsystem shall integrate heterogeneous GPU/NPU hardware providing a total processing capacity of 275 TOPS (including 32 TOPS dedicated tensor cores) and 64GB RAM via an Nvidia Jetson Orin Industrial SOM.</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -2007,22 +1990,22 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Embedded Avionics Hardware</t>
+          <t>Embedded Compute Hardware</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Section 4 (Domain 4), Section 6.2 (p. 5, 7)</t>
+          <t>Section 1.1, Section 6.1, Section 11.2 (p. 1, 6, 11)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Hardware layer explicitly designates 'Dedicated 32-bit automotive/aerospace microcontrollers managing low-latency inner attitude loops'.</t>
+          <t>Specifications mandate 'Nvidia Jetson Orin Industrial SOM (64GB RAM, 275 TOPS compute rating)' with 32 TOPS tensor blocks.</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -2042,24 +2025,24 @@
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>Specific microcontroller part number (e.g. STM32H753), core operating clock frequency, and memory capacity not defined.</t>
+          <t>SOM operating power dissipation profile (e.g. 40W vs 60W mode) under high-altitude low air density cooling not stated.</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>Baseline embedded processor architecture.</t>
+          <t>Explicit hardware specifications in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-P-007</t>
+          <t>DRAFT-P-008</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>The system shall satisfy tactical flight envelope performance thresholds for maximum takeoff weight (MTOW), payload capacity, endurance, operating ceiling, and wind resistance in high-altitude mountain theaters.</t>
+          <t>Onboard PyTorch visual neural models compiled via TensorRT 8.5 for 8-bit quantization (INT8) shall achieve real-time inference execution at a throughput of 60 frames per second (60 FPS).</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2069,22 +2052,22 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Aerodynamics &amp; Flight Envelope</t>
+          <t>Edge AI Optimization</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0 &amp; P01_Project_Scope_Baseline.md</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Section 1.4, Section 2.1 (p. 2, 3); Scope Baseline Sec 10, 12</t>
+          <t>Section 6.1 (TensorRT Acceleration), Section 6.2 (p. 6)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Platform is engineered for Ladakh and Siachen mountain frontiers, but specific numerical aerodynamic thresholds are omitted from overview.</t>
+          <t>Explicitly specifies 'PyTorch visual neural models compiled via TensorRT for 8-bit quantized low-latency inferencing at 60 FPS'.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2097,31 +2080,31 @@
           <t>Test</t>
         </is>
       </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Numerical values for MTOW (kg), payload mass (kg), flight endurance (hours), service ceiling (m AMSL), and wind shear resistance (knots) must be provided from master proposal.</t>
+          <t>Input image resolution at 60 FPS (e.g. 640x640 vs 1080p) and inference batch size need confirmation.</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>Recorded as Open Question QUE-SCP-002 and Assumption ASM-ENG-002.</t>
+          <t>Explicit numerical framerate in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-P-008</t>
+          <t>DRAFT-P-009</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>The onboard neural network models for semantic segmentation, temporal change detection, and super-resolution shall be compiled and executed using INT8 post-training quantization via NVIDIA TensorRT.</t>
+          <t>The faceted carbon monocoque airframe with embedded radar-absorbing material (RAM) shall exhibit an estimated Radar Cross-Section (RCS) of less than 0.01 m² (&lt; 0.01 m²) across X and Ku radar frequency bands.</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -2131,22 +2114,22 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Edge AI Optimization</t>
+          <t>Stealth &amp; Signature Control</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Section 5.2 (Stage 3), Section 6.3 (p. 6, 7)</t>
+          <t>Section 2.2 (Objective Pillars) (p. 2)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Software stack mandates PyTorch pipeline exported to ONNX and compiled via NVIDIA TensorRT for INT8 post-training quantization.</t>
+          <t>Explicitly specifies 'Faceted radar-absorbing airframe yielding an estimated RCS &lt; 0.01 m² across X and Ku radar bands'.</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -2156,7 +2139,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -2166,49 +2149,49 @@
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>Maximum allowable neural accuracy degradation percentage resulting from INT8 quantization vs FP32 baseline not stated.</t>
+          <t>Specific azimuth and elevation aspect angle cones for the &lt;0.01 m² RCS threshold not detailed.</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>Defines computational optimization format for edge AI engines.</t>
+          <t>Explicit numerical threshold in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-S-001</t>
+          <t>DRAFT-P-010</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>The system shall execute the PX4 flight stabilization stack on a dedicated bare-metal microcontroller physically and electrically isolated from the Linux edge compute operating system.</t>
+          <t>The Software-Defined Radio (SDR) subsystem shall operate across a continuous wideband radio frequency monitoring range spanning from 10 MHz to 6 GHz.</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Architectural Isolation &amp; Airworthiness</t>
+          <t>Electronic Warfare Spectrum</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Section 8.3 (Asynchronous Thread Isolation) (p. 9)</t>
+          <t>Section 4 (DSP Domain), Section 7 (Module 04) (p. 4, 7)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>The PX4 flight stabilization stack executes on a dedicated bare-metal microcontroller independent of the Linux edge compute operating system.</t>
+          <t>Explicitly specifies 'wideband SDR spectrum streams (10 MHz - 6 GHz)' and Module 04 RF antenna inputs.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2218,7 +2201,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Inspection</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -2228,24 +2211,24 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>None. Confirmed architectural requirement.</t>
+          <t>Tuning step size, frequency switching speed, and receiver noise figure across 10 MHz–6 GHz not defined.</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Guarantees that high-level AI faults or kernel crashes cannot compromise core flight safety.</t>
+          <t>Explicit frequency range in blueprint.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-S-002</t>
+          <t>DRAFT-S-001</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>The system flight controller shall autonomously maintain mission execution, waypoint navigation, attitude hold, or return-to-home (RTH) without degradation in the event of an edge AI process exception, crash, or memory thrashing.</t>
+          <t>The system flight control software shall execute on dedicated bare-metal ARM Cortex-M7 processors physically independent of the Linux Edge-AI compute module to ensure that edge software crashes cannot affect flight stability.</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -2255,22 +2238,22 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Failsafe &amp; Fault Tolerance</t>
+          <t>Architectural Isolation &amp; Airworthiness</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Section 8.3 (Zero-Overhead Watchdog) (p. 9)</t>
+          <t>Section 8.2 (Asynchronous Hardware Firewall) (p. 8)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>If an edge AI model experiences an exception or memory thrashing, the primary autopilot continues mission execution, waypoint navigation, or return-to-home without degradation.</t>
+          <t>Explicitly specifies 'The flight control system runs on dedicated bare-metal ARM Cortex-M7 processors physically independent of the Linux Edge-AI compute module.'</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -2280,7 +2263,7 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Inspection</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -2290,24 +2273,24 @@
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Autopilot heartbeat timeout duration (milliseconds) before declaring edge compute link loss needs formal confirmation.</t>
+          <t>None. Confirmed architectural requirement.</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>Critical fail-safe architectural isolation protocol.</t>
+          <t>Prevents AI process exceptions from compromising core flight stabilization.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-S-003</t>
+          <t>DRAFT-S-002</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The system shall interlock cargo drop mechanisms and authorized payload actuation circuits via opto-isolated solid-state I/O requiring dual-redundant discrete logic signals to prevent uncommanded release during boot or fault states.</t>
+          <t>The system flight software lifecycle and airborne electronic hardware components shall comply with DO-178C (software) and DO-254 (airborne electronic hardware) safety and airworthiness standards.</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2317,22 +2300,22 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Effector &amp; Payload Interlocking</t>
+          <t>Safety Certification &amp; Compliance</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Section 8.2, Section 8.3 (p. 9)</t>
+          <t>Section 4 (Systems Safety) (p. 4)</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Table 8.2 mandates 'Dual-Redundant Discrete Logic Signals' and 'Hardware interlock preventing uncommanded release during boot or fault conditions'.</t>
+          <t>Systems Safety discipline explicitly 'Manages DO-178C and DO-254 compliance tracking, hardware stress testing, and emergency return modes.'</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -2342,7 +2325,7 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Inspection</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2352,24 +2335,24 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Logic voltage levels, arming state sequence, and hardware reset default state need formal definition in Interface Control Document (ICD).</t>
+          <t>Specific Design Assurance Level (DAL A, B, or C) allocation across subsystems needs formal publication in PSAC/PHAC.</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>Module 06 and Layer G safety control.</t>
+          <t>Military and civil aviation certification baseline.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-S-004</t>
+          <t>DRAFT-S-003</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>The flight control system shall continuously monitor hardware watchdog heartbeats from the edge compute module over UART/Ethernet and automatically execute internal failsafe procedures upon link loss.</t>
+          <t>The system shall route autopilot-to-compute telemetry over redundant CAN-BUS 2.0B interfaces with hardware watchdog heartbeats, automatically executing internal failsafe procedures upon communication loss.</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -2379,22 +2362,22 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Communication Failsafe</t>
+          <t>Failsafe &amp; Fault Tolerance</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Section 8.2 (Autopilot to Compute Interface) (p. 9)</t>
+          <t>Section 6.2, Section 8.1 (p. 6, 8)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Table 8.2 specifies 'Hardware watchdog heartbeats; automatic fallback to internal failsafe on link loss'.</t>
+          <t>Specifies redundant CAN-BUS micro-XRCE agents with 'Hardware watchdog heartbeats with auto-failsafe fallback.'</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -2414,24 +2397,24 @@
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>Specific sequence of internal failsafe actions (hover in place vs dead-reckoning RTH vs controlled landing) not specified in source.</t>
+          <t>CAN-BUS baud rate and watchdog timeout window (milliseconds) before declaring link loss need definition.</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Prevents loss of control if inter-processor communication drops.</t>
+          <t>High-reliability fault-tolerant bus protocol.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-S-005</t>
+          <t>DRAFT-S-004</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>The system shall physically isolate Software-Defined Radio (SDR) RF ingress circuits from flight motor lines and ESC power electronics using strict electromagnetic interference (EMI) gaskets and shielding.</t>
+          <t>The AeroDrop cargo release mechanism shall be controlled via opto-isolated solid-state discrete I/O requiring dual high/low logic signals to prevent accidental payload drops during boot or fault states.</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2441,22 +2424,22 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>EMI / EMC Isolation</t>
+          <t>Effector &amp; Payload Interlocking</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Section 8.2 (SDR RF Ingress Interface) (p. 9)</t>
+          <t>Section 8.1 (Interface Vector: Cargo Release) (p. 8)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Table 8.2 specifies 'Strict RF shielding (EMI gaskets) isolating RF circuits from flight motor lines'.</t>
+          <t>Table 8.1 mandates 'Opto-Isolated Discrete I/O', 'Dual High/Low Logic', and 'Dual-redundant interlocks preventing accidental payload drop.'</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2466,7 +2449,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Inspection</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2476,24 +2459,24 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Target shielding attenuation (dB) and applicable military EMC standard (e.g. MIL-STD-461) not specified in overview.</t>
+          <t>Discrete logic voltage thresholds and hardware interlock disarm timeout need definition.</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Prevents high-current propulsion switching noise from blinding RF receivers.</t>
+          <t>Module 06 and Layer G safety control.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>DRAFT-S-006</t>
+          <t>DRAFT-S-005</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>The system edge compute software architecture shall restrict all inter-process communications to local shared memory (POSIX shm) or loopback Unix domain sockets, enforcing physical and logical prohibitions against unvetted external network bridging.</t>
+          <t>The system edge compute software architecture shall restrict all inter-process communications to local shared memory IPC queues under an air-gapped Vanguard-Linux OS, with complete prohibition of unvetted external network bridging.</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -2508,17 +2491,17 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Section 8.3 (Air-Gapped Local Network) (p. 9)</t>
+          <t>Section 6.1, Section 6.2 (p. 6)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Specifies 'All inter-process communication occurs over local shared memory (POSIX shm) or loopback Unix sockets, with physical and logical prohibitions against unvetted external connections'.</t>
+          <t>Ecosystem specifies 'Air-gapped Vanguard-Linux OS with real-time PREEMPT_RT patches' and 'isolated ROS 2 Humble nodes via shared memory IPC queues.'</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -2543,19 +2526,19 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>Protects avionics and AI models from remote network ingress and data exfiltration.</t>
+          <t>Prevents unauthorized remote network infiltration.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>DRAFT-S-007</t>
+          <t>DRAFT-S-006</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>No system software module or hardware subsystem shall progress to physical flight testing without documented testbench validation logs and formal stage gate sign-off across preceding tiers of the 10-Tier Validation Ladder.</t>
+          <t>The system avionics and inter-module buses shall sustain continuous operation for at least 48 hours with zero bus collisions during benchtop integration (Tier 4) prior to receiving authorization for flight testing.</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2570,17 +2553,17 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Section 10.1, Section 10.2 (p. 11)</t>
+          <t>Section 10 (Tier 4 Exit Criteria) (p. 10)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Mandates 'Verification Before Progression: No subsystem enters flight testing without validated testbench logs and formal gate sign-offs.'</t>
+          <t>Tier 4 Benchtop Integration explicitly establishes exit criteria as 'Zero bus collisions over 48h.'</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2590,7 +2573,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Inspection</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2600,12 +2583,12 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Stage gate review authority committee composition and sign-off criteria for Tiers 1–5 need formal definition in project QA plan.</t>
+          <t>Definition of bus collision logging mechanism and acceptable bus utilization percentage not specified.</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>Prevents untested software or hardware from flying on physical airframes.</t>
+          <t>Explicit testing gate in blueprint.</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2600,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>The engineering team shall author, baseline, and freeze a formal System Requirements Specification (SRS) governing all 20 frozen capabilities prior to the completion of Milestone 1 (Month 4).</t>
+          <t>The engineering team shall baseline and freeze the comprehensive System Requirements Specification (SRS) governing all 18 core subsystems during Milestone 1 (Months 1–4).</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
@@ -2632,17 +2615,17 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Section 9.2 (Milestone 1 Activities) (p. 10)</t>
+          <t>Executive Summary, Section 9.1 (p. 0/1, 9)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Milestone 1 mandates 'Freeze System Requirements Specification (SRS)' across Months 1–4.</t>
+          <t>Milestone 1 mandates Digital Twin and software simulation freeze across Months 1–4.</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -2662,12 +2645,12 @@
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>SRS structure standard (e.g. ISO/IEC/IEEE 29148) and formal customer approval timeline not stated.</t>
+          <t>SRS format standard (IEEE 29148) and formal customer approval cycle need confirmation.</t>
         </is>
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>Governs transition from Milestone 1 to Milestone 2.</t>
+          <t>Milestone 1 deliverable.</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2662,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Every software module, hardware component specification, and verification test case shall maintain bidirectional traceability mapped directly to the frozen iDEX contract deliverables (D1 through D20).</t>
+          <t>The engineering team shall maintain a configuration-controlled Project Scope Baseline document establishing system boundaries, subsystem decomposition, constraints, and open scope decisions.</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2689,22 +2672,22 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Traceability &amp; Compliance</t>
+          <t>Configuration &amp; Scope Management</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>Task Order TRAIN-002 &amp; P01_Project_Scope_Baseline.md</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Section 10.2 (Requirement Traceability) (p. 11)</t>
+          <t>Task Order Sec 1, Sec 4; Scope Baseline Sec 1</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Explicitly mandates 'Requirement Traceability: Every software module and hardware spec maps directly to frozen iDEX deliverables (D1 through D20).'</t>
+          <t>Mandated deliverable under Task Order TRAIN-002 on 22 October 2026.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2717,19 +2700,19 @@
           <t>Inspection</t>
         </is>
       </c>
-      <c r="J34" s="9" t="inlineStr">
-        <is>
-          <t>Pending Clarification</t>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>The itemized list of 20 deliverables (D1 through D20) must be released from the master iDEX proposal annex.</t>
+          <t>None. Delivered as P01_Project_Scope_Baseline.md.</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>Recorded as Assumption ASM-ENG-001 and Question QUE-SCP-001 in Task 1.</t>
+          <t>Deliverable 1 under Task Order TRAIN-002.</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2724,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>The engineering team shall maintain a configuration-controlled Project Scope Baseline document establishing system boundaries, PECLF allocations, constraints, and open scope decisions.</t>
+          <t>The engineering team shall deliver an auditable, structured Initial Requirements Register workbook categorizing functional, performance, safety, and documentation requirements on 22 October 2026.</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -2756,12 +2739,12 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Task Order TRAIN-002 &amp; P01_Project_Scope_Baseline.md</t>
+          <t>Task Order TRAIN-002</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Task Order Sec 1, Sec 4; Scope Baseline Sec 1 (p. 1)</t>
+          <t>Task Order Sec 1, Sec 2, Sec 5</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2786,12 +2769,12 @@
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>None. Delivered as P01_Project_Scope_Baseline.md.</t>
+          <t>None. Delivered as P02_Initial_Requirements_Register.xlsx.</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>Deliverable 1 under Task Order TRAIN-002.</t>
+          <t>Deliverable 2 under Task Order TRAIN-002.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2786,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>The engineering team shall deliver an auditable, structured Initial Requirements Register workbook categorizing functional, performance, safety, and documentation requirements on 22 October 2026.</t>
+          <t>The engineering team shall establish and maintain life-cycle data artifacts, requirement-to-code traceability, and verification evidence complying with DO-178C and DO-254 development standards.</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2813,22 +2796,22 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Configuration &amp; Scope Management</t>
+          <t>Certification &amp; Traceability</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Task Order TRAIN-002</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Task Order Sec 1, Sec 2, Sec 5</t>
+          <t>Section 4 (Systems Safety) (p. 4)</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Mandated deliverable under Task Order TRAIN-002 on 22 October 2026.</t>
+          <t>Mandates DO-178C and DO-254 compliance tracking and requirement traceability.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2848,12 +2831,12 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>None. Work authorized under TRAIN-002.</t>
+          <t>Selection of formal requirements management and traceability tool (e.g. Polarion / DOORS) needs project sign-off.</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>Current deliverable (P02_Initial_Requirements_Register.xlsx).</t>
+          <t>Core safety certification documentation.</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2848,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>All software source code commits, firmware releases, and hardware schematic promotions shall occur exclusively through peer-reviewed, cryptographically signed internal repository branches.</t>
+          <t>The engineering team shall compile formal test reports, bus collision audit logs over 48 hours, and sub-zero thermal profiling down to -30°C for all integrated benchtop HIL avionics during Milestone 2.</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -2875,22 +2858,22 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Configuration &amp; Quality Assurance</t>
+          <t>Test &amp; Verification Reporting</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Section 10.2 (Controlled Integration) (p. 11)</t>
+          <t>Section 9.1, Section 10 (Tier 4, Tier 5) (p. 9, 10)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Explicitly states 'Controlled Integration: Code and hardware promotions occur exclusively through peer-reviewed, cryptographically signed internal repository branches.'</t>
+          <t>Milestone 2 deliverables and Tiers 4/5 require documented testbed verification logs and thermal chamber reports.</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
@@ -2910,12 +2893,12 @@
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>Cryptographic signing key management policy (GPG key length/storage) and CI/CD promotion gate rules need documentation.</t>
+          <t>Test reporting template and power margin thresholds need formalization in HIL Test Plan.</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>Core engineering integrity protocol.</t>
+          <t>Milestone 2 documentation deliverable.</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2910,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>The project team shall compile comprehensive iDEX demonstration dossiers, safety registers, failure mode analyses, and manufacturing documentation packages prior to Milestone 5 pre-induction field evaluation.</t>
+          <t>The project team shall compile comprehensive defense qualification dossiers, safety registers, failure mode analyses, and manufacturing documentation packages prior to Milestone 5 pre-induction field trials.</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2942,17 +2925,17 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
+          <t>AVT-AETH-2026-X9</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Section 9.2 (Milestone 5 Outputs) (p. 10)</t>
+          <t>Section 9.1 (Milestone 5), Section 10 (Tier 10) (p. 9, 10)</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Milestone 5 deliverables include 'comprehensive iDEX demonstration dossiers, safety registers, and manufacturing documentation' for MoD evaluators.</t>
+          <t>Milestone 5 deliverables mandate field evaluation dossiers and complete mission gate success records for defense evaluators.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2972,7 +2955,7 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Specific MoD evaluation dossier format and safety case standard (e.g. Def Stan 00-056 or equivalent) not detailed.</t>
+          <t>Defense evaluation authority dossier formatting guidelines not detailed.</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -2981,75 +2964,13 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>DRAFT-D-007</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>The engineering team shall document formal power consumption audits and thermal profiling test reports down to -20°C for all integrated benchtop HIL avionics and compute modules during Milestone 2.</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Test &amp; Verification Reporting</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Section 9.2 (Milestone 2 Outputs) (p. 10)</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>Milestone 2 deliverables explicitly mandate 'power/thermal audit reports, and verified inter-module communication drivers.'</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>Not Assigned</t>
-        </is>
-      </c>
-      <c r="I39" s="8" t="inlineStr">
-        <is>
-          <t>Inspection</t>
-        </is>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>Proposed for Review</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>Power budget allocation breakdown and thermal reporting template need formal definition in Milestone 2 test plan.</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>Milestone 2 documentation deliverable.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L39"/>
+  <autoFilter ref="A1:L38"/>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Category" error="Your entry is not valid" promptTitle="Category" prompt="Please select from the list" type="list">
+    <dataValidation sqref="C2:C38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Functional,Performance,Safety,Documentation"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Status" error="Your entry is not valid" promptTitle="Status" prompt="Please select from the list" type="list">
+    <dataValidation sqref="J2:J38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draft,Pending Clarification,Proposed for Review"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3073,16 +2994,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>RUDRAEDGE RE-T1 (SPECTRA) — REQUIREMENTS REGISTER SUMMARY</t>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>AEROVANGUARD AV-X9 AETHERIS (BLOCK II) — REQUIREMENTS REGISTER SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Project Reference: RE-iDEX-PROPOSAL-2026-R1 | Task Order: TRAIN-002 | Date: 22 October 2026 | Engineer: Priyanka Sharma</t>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Project Reference: AVT-MOD-PROP-2026-R4 | Task Order: TRAIN-002 | Date: 22 October 2026 | Engineer: Priyanka Sharma</t>
         </is>
       </c>
     </row>
@@ -3110,100 +3031,100 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="B5" s="13">
-        <f>COUNTIF(Requirements_Register!C2:C39, "Functional")</f>
+      <c r="B5" s="12">
+        <f>COUNTIF(Requirements_Register!C2:C38, "Functional")</f>
         <v/>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="13">
         <f>B5/$B$9</f>
         <v/>
       </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>Core platform behaviors, sensor data acquisition, edge AI inference, FSO communications, and navigation logic.</t>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Core platform behaviors, 4K/LWIR sensor ingestion, AetherNav VIO, AeroCore AI, AetherBeam laser, and AeroDrop release.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="B6" s="13">
-        <f>COUNTIF(Requirements_Register!C2:C39, "Performance")</f>
+      <c r="B6" s="12">
+        <f>COUNTIF(Requirements_Register!C2:C38, "Performance")</f>
         <v/>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="13">
         <f>B6/$B$9</f>
         <v/>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Measurable engineering thresholds including latency (&lt;1ms), operating temp (-20°C), RF frequency bands (400MHz-6GHz), and drift limits.</t>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Documented engineering thresholds: &lt;250 µs latency, 6,500m ceiling, 25 m/s wind shear, -30°C cold, &lt;0.8m/hr drift, 1.2 Gbps/18km FSO, 275 TOPS Orin SOM, 60 FPS.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="B7" s="13">
-        <f>COUNTIF(Requirements_Register!C2:C39, "Safety")</f>
+      <c r="B7" s="12">
+        <f>COUNTIF(Requirements_Register!C2:C38, "Safety")</f>
         <v/>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="13">
         <f>B7/$B$9</f>
         <v/>
       </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>Flight-critical isolation firewalls, bare-metal PX4 decoupling, watchdog timers, hardware effector interlocks, and air-gapped networking.</t>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Hardware firewalls, bare-metal STM32H7 isolation, DO-178C/DO-254 safety compliance, redundant CAN-BUS watchdog, and 48h zero-collision testing.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="B8" s="13">
-        <f>COUNTIF(Requirements_Register!C2:C39, "Documentation")</f>
+      <c r="B8" s="12">
+        <f>COUNTIF(Requirements_Register!C2:C38, "Documentation")</f>
         <v/>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="13">
         <f>B8/$B$9</f>
         <v/>
       </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>Mandated project artifacts, SRS baselining (M1), deliverable traceability (D1-D20), cryptographic commit signing, and audit dossiers.</t>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Mandated project artifacts, SRS freeze (M1), DO-178C/DO-254 traceability, HIL test reports, and defense qualification dossiers.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Total Requirements Count</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="16">
         <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="17">
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Complete count of all draft requirement records captured in initial register.</t>
         </is>
@@ -3211,102 +3132,102 @@
     </row>
     <row r="10" ht="16" customHeight="1"/>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Status Breakdown</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Percentage of Total</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Status Definition &amp; Action Required</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Proposed for Review</t>
-        </is>
-      </c>
-      <c r="B12" s="13">
-        <f>COUNTIF(Requirements_Register!J2:J39, "Proposed for Review")</f>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Proposed for Review</t>
+        </is>
+      </c>
+      <c r="B12" s="12">
+        <f>COUNTIF(Requirements_Register!J2:J38, "Proposed for Review")</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="13">
         <f>B12/$B$9</f>
         <v/>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>Sufficient source evidence exists; ready for peer review by Chief Systems Engineer.</t>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Grounded in technical blueprint AVT-AETH-2026-X9; ready for internal review by Chief Systems Architect.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Pending Clarification</t>
         </is>
       </c>
-      <c r="B13" s="13">
-        <f>COUNTIF(Requirements_Register!J2:J39, "Pending Clarification")</f>
+      <c r="B13" s="12">
+        <f>COUNTIF(Requirements_Register!J2:J38, "Pending Clarification")</f>
         <v/>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="13">
         <f>B13/$B$9</f>
         <v/>
       </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>Requirement identified from source, but numerical threshold, protocol, or interface specification is missing.</t>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Requirement identified from source, but detailed protocol or interface specification is pending.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="B14" s="13">
-        <f>COUNTIF(Requirements_Register!J2:J39, "Draft")</f>
+      <c r="B14" s="12">
+        <f>COUNTIF(Requirements_Register!J2:J38, "Draft")</f>
         <v/>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="13">
         <f>B14/$B$9</f>
         <v/>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Initial draft requirement entry under active authoring.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Total Categorized by Status</t>
         </is>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="16">
         <f>SUM(B12:B14)</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="17">
         <f>SUM(C12:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Matches total count of primary requirements register.</t>
         </is>
@@ -3382,34 +3303,34 @@
           <t>SRC-01</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>RudraEdge RE-T1 (Spectra) Project Introduction &amp; Technical Overview: Understanding the System • Technology • Architecture • Development</t>
-        </is>
-      </c>
-      <c r="C2" s="20" t="inlineStr">
-        <is>
-          <t>REA-T1-OVERVIEW-2026-V1.0</t>
-        </is>
-      </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>AV-X9 Aetheris Platform: Project Introduction &amp; System Architecture Overview</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>AVT-AETH-2026-X9</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>Version 1.0 (2026)</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>Sections 1 through 11 (Pages 1–12)</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>Primary engineering source for platform concept, 8-layer PECLF framework, 20 frozen capabilities, 10-Tier Validation Ladder, 18-month phased engineering lifecycle, interface buses, and architectural isolation firewalls.</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>Lacks itemized descriptions for deliverables D1 through D20; omits specific numerical flight performance envelope thresholds (MTOW, endurance, operating ceiling, payload capacity in kg).</t>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Primary engineering blueprint: 8-layer PECLF framework, 18 core subsystems, 10-Tier Verification Ladder, 18-month phased lifecycle, exact flight thresholds (6,500m ceiling, 25 m/s wind shear, -30°C cold), &lt;250 µs latency, 1550nm 1.2 Gbps FSO link (18 km), 275 TOPS Orin Industrial SOM, and DO-178C/DO-254 standards.</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Exact numerical Maximum Takeoff Weight (MTOW) and cargo payload mass in kg omitted from unclassified overview.</t>
         </is>
       </c>
     </row>
@@ -3419,34 +3340,34 @@
           <t>SRC-02</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>Project Scope Baseline: RudraEdge RE-T1 (Spectra) Tactical UAS</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Project Scope Baseline: AeroVanguard AV-X9 Aetheris (Block II) Tactical UAS</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>P01_Project_Scope_Baseline.md</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Version 0.1 (22 October 2026)</t>
-        </is>
-      </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Version 0.2 (22 October 2026)</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>Sections 1 through 15 (Complete Document)</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr">
-        <is>
-          <t>System boundaries, PECLF subsystem scope allocation, in-scope vs. out-of-scope boundaries, active project constraints register, assumptions register, inter-module interface dependencies, and open scope questions.</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="inlineStr">
-        <is>
-          <t>Internal engineering baseline document drafted under Task TRAIN-002; pending formal steering committee and peer review approval.</t>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>System boundaries, 18 subsystem scope allocation, in-scope vs. out-of-scope boundaries, active project constraints register, assumptions register, inter-module interface standards, and open scope questions.</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Internal engineering baseline document drafted under Task TRAIN-002; pending formal peer review approval.</t>
         </is>
       </c>
     </row>
@@ -3456,32 +3377,32 @@
           <t>SRC-03</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Task Order: Requirements Baseline (TRAIN-002)</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>TRAIN-002</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>22 October 2026</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Sections 1 through 11</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Engineer assignment (Priyanka Sharma, Systems Requirements &amp; Configuration Engineer), task authorization boundaries, deliverable specifications (P01 and P02), workbook formatting guidelines, and training expenditure constraints.</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>Authorized scope is strictly bounded to desk-based systems engineering, requirements modeling, and documentation; explicitly excludes physical hardware procurement, live flight tests, and paid cloud services.</t>
         </is>

</xml_diff>